<commit_message>
Spatial Visualisasi, pemetaan cluster
</commit_message>
<xml_diff>
--- a/Kompilasi Data 2.xlsx
+++ b/Kompilasi Data 2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22527"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DINDA\Documents\datmin asekk\fix bgt\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maeli\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A5095E6-70F0-4AF4-A02E-18F458D09B5A}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{EA46FAB0-AD03-4E93-B93F-40C73726C29F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{3F342D85-5833-46D0-AAAB-3415AE56ECD8}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{3F342D85-5833-46D0-AAAB-3415AE56ECD8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="52">
   <si>
     <t>Provinsi</t>
   </si>
@@ -178,14 +178,24 @@
   </si>
   <si>
     <t>D.I. Yogyakarta</t>
+  </si>
+  <si>
+    <t>Makanan Per Kapita</t>
+  </si>
+  <si>
+    <t>Non Makanan Per Kapita</t>
+  </si>
+  <si>
+    <t>Persentase Penduduk Miskin - September</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -203,20 +213,27 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12"/>
+      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="5">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -239,52 +256,21 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" indent="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma 2" xfId="1" xr:uid="{170AE5E6-737D-4E19-8113-D14D742B2F6C}"/>
@@ -304,9 +290,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -344,7 +330,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -450,7 +436,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -592,7 +578,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -600,1380 +586,1735 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6669FCC6-6420-481B-B6E4-E94222D70C7F}">
-  <dimension ref="A1:K39"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:N39"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="23.21875" customWidth="1"/>
-    <col min="3" max="3" width="15.109375" customWidth="1"/>
-    <col min="5" max="5" width="17.6640625" customWidth="1"/>
-    <col min="6" max="6" width="12.77734375" customWidth="1"/>
+    <col min="1" max="1" width="23.1796875" customWidth="1"/>
+    <col min="3" max="3" width="15.08984375" customWidth="1"/>
+    <col min="5" max="5" width="17.6328125" customWidth="1"/>
+    <col min="6" max="6" width="12.81640625" customWidth="1"/>
     <col min="7" max="7" width="12" customWidth="1"/>
-    <col min="9" max="9" width="16.77734375" customWidth="1"/>
+    <col min="9" max="9" width="16.81640625" customWidth="1"/>
+    <col min="11" max="11" width="17.6328125" customWidth="1"/>
+    <col min="12" max="12" width="17.54296875" customWidth="1"/>
+    <col min="13" max="13" width="21.453125" customWidth="1"/>
+    <col min="14" max="14" width="35.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="L1" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="1">
         <v>74.03</v>
       </c>
-      <c r="C2">
+      <c r="C2" s="1">
         <v>98.864333947206873</v>
       </c>
-      <c r="D2" s="3">
+      <c r="D2" s="2">
         <v>50.5</v>
       </c>
       <c r="E2" s="1">
         <v>37.65</v>
       </c>
-      <c r="F2">
+      <c r="F2" s="1">
         <v>108507</v>
       </c>
-      <c r="G2">
+      <c r="G2" s="1">
         <v>5086801</v>
       </c>
-      <c r="H2" s="4">
+      <c r="H2" s="1">
         <v>75.989999999999995</v>
       </c>
-      <c r="I2" s="2">
+      <c r="I2" s="3">
         <v>5.12</v>
       </c>
-      <c r="J2">
+      <c r="J2" s="1">
         <v>198.69</v>
       </c>
-      <c r="K2">
+      <c r="K2" s="1">
         <v>0.99</v>
       </c>
-    </row>
-    <row r="3" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="L2" s="4">
+        <v>722434.00079302699</v>
+      </c>
+      <c r="M2" s="4">
+        <v>542298.94524701172</v>
+      </c>
+      <c r="N2" s="1">
+        <v>12.64</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="1">
         <v>74.02</v>
       </c>
-      <c r="C3">
+      <c r="C3" s="1">
         <v>96.613773924423356</v>
       </c>
-      <c r="D3" s="3">
+      <c r="D3" s="2">
         <v>49.05</v>
       </c>
       <c r="E3" s="1">
         <v>35.380000000000003</v>
       </c>
-      <c r="F3">
+      <c r="F3" s="1">
         <v>123911</v>
       </c>
-      <c r="G3">
+      <c r="G3" s="1">
         <v>7957689</v>
       </c>
-      <c r="H3" s="4">
+      <c r="H3" s="1">
         <v>73.150000000000006</v>
       </c>
-      <c r="I3" s="6">
+      <c r="I3" s="3">
         <v>2.72</v>
       </c>
-      <c r="J3">
+      <c r="J3" s="1">
         <v>172.37</v>
       </c>
-      <c r="K3">
+      <c r="K3" s="1">
         <v>4.0600000000000005</v>
       </c>
-    </row>
-    <row r="4" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+      <c r="L3" s="4">
+        <v>734270.16389291186</v>
+      </c>
+      <c r="M3" s="4">
+        <v>606687.15052857681</v>
+      </c>
+      <c r="N3" s="1">
+        <v>7.19</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="1">
         <v>74.489999999999995</v>
       </c>
-      <c r="C4">
+      <c r="C4" s="1">
         <v>98.055987558320368</v>
       </c>
-      <c r="D4" s="3">
+      <c r="D4" s="2">
         <v>47.62</v>
       </c>
       <c r="E4" s="1">
         <v>28.75</v>
       </c>
-      <c r="F4">
+      <c r="F4" s="1">
         <v>88053</v>
       </c>
-      <c r="G4">
+      <c r="G4" s="1">
         <v>4567033</v>
       </c>
-      <c r="H4" s="4">
+      <c r="H4" s="1">
         <v>75.14</v>
       </c>
-      <c r="I4" s="6">
+      <c r="I4" s="3">
         <v>5.56</v>
       </c>
-      <c r="J4">
+      <c r="J4" s="1">
         <v>194.63000000000002</v>
       </c>
-      <c r="K4">
+      <c r="K4" s="1">
         <v>3.0799999999999996</v>
       </c>
-    </row>
-    <row r="5" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+      <c r="L4" s="4">
+        <v>797727.89179974352</v>
+      </c>
+      <c r="M4" s="4">
+        <v>683125.28766400262</v>
+      </c>
+      <c r="N4" s="1">
+        <v>5.42</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="1">
         <v>74.790000000000006</v>
       </c>
-      <c r="C5">
+      <c r="C5" s="1">
         <v>98.395721925133699</v>
       </c>
-      <c r="D5" s="3">
+      <c r="D5" s="2">
         <v>47.42</v>
       </c>
       <c r="E5" s="1">
         <v>36.93</v>
       </c>
-      <c r="F5">
+      <c r="F5" s="1">
         <v>54425</v>
       </c>
-      <c r="G5">
+      <c r="G5" s="1">
         <v>3494581</v>
       </c>
-      <c r="H5" s="4">
+      <c r="H5" s="1">
         <v>82.49</v>
       </c>
-      <c r="I5" s="6">
+      <c r="I5" s="3">
         <v>2.57</v>
       </c>
-      <c r="J5">
+      <c r="J5" s="1">
         <v>156.56</v>
       </c>
-      <c r="K5">
+      <c r="K5" s="1">
         <v>5.66</v>
       </c>
-    </row>
-    <row r="6" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
+      <c r="L5" s="4">
+        <v>824229.25418610033</v>
+      </c>
+      <c r="M5" s="4">
+        <v>738936.22511853394</v>
+      </c>
+      <c r="N5" s="1">
+        <v>6.36</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B6">
+      <c r="B6" s="1">
         <v>73.430000000000007</v>
       </c>
-      <c r="C6">
+      <c r="C6" s="1">
         <v>98.296529968454266</v>
       </c>
-      <c r="D6" s="3">
+      <c r="D6" s="2">
         <v>47.1</v>
       </c>
       <c r="E6" s="1">
         <v>33.9</v>
       </c>
-      <c r="F6">
+      <c r="F6" s="1">
         <v>31268</v>
       </c>
-      <c r="G6">
+      <c r="G6" s="1">
         <v>2065021</v>
       </c>
-      <c r="H6" s="4">
+      <c r="H6" s="1">
         <v>85.91</v>
       </c>
-      <c r="I6" s="6">
+      <c r="I6" s="3">
         <v>3.65</v>
       </c>
-      <c r="J6">
+      <c r="J6" s="1">
         <v>150.79999999999998</v>
       </c>
-      <c r="K6">
+      <c r="K6" s="1">
         <v>4.12</v>
       </c>
-    </row>
-    <row r="7" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+      <c r="L6" s="4">
+        <v>773667.40659423242</v>
+      </c>
+      <c r="M6" s="4">
+        <v>698833.34572358232</v>
+      </c>
+      <c r="N6" s="1">
+        <v>7.26</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B7">
+      <c r="B7" s="1">
         <v>72.3</v>
       </c>
-      <c r="C7">
+      <c r="C7" s="1">
         <v>99.147121535181242</v>
       </c>
-      <c r="D7" s="3">
+      <c r="D7" s="2">
         <v>46.66</v>
       </c>
       <c r="E7" s="1">
         <v>37.840000000000003</v>
       </c>
-      <c r="F7">
+      <c r="F7" s="1">
         <v>77678</v>
       </c>
-      <c r="G7">
+      <c r="G7" s="1">
         <v>6321594</v>
       </c>
-      <c r="H7" s="4">
+      <c r="H7" s="1">
         <v>74.62</v>
       </c>
-      <c r="I7" s="6">
+      <c r="I7" s="3">
         <v>1.96</v>
       </c>
-      <c r="J7">
+      <c r="J7" s="1">
         <v>184.64</v>
       </c>
-      <c r="K7">
+      <c r="K7" s="1">
         <v>9.34</v>
       </c>
-    </row>
-    <row r="8" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
+      <c r="L7" s="4">
+        <v>711510.48106993677</v>
+      </c>
+      <c r="M7" s="4">
+        <v>577490.47027720732</v>
+      </c>
+      <c r="N7" s="1">
+        <v>10.51</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A8" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B8">
+      <c r="B8" s="1">
         <v>73.39</v>
       </c>
-      <c r="C8">
+      <c r="C8" s="1">
         <v>99.075297225891674</v>
       </c>
-      <c r="D8" s="3">
+      <c r="D8" s="2">
         <v>46.07</v>
       </c>
       <c r="E8" s="1">
         <v>39.6</v>
       </c>
-      <c r="F8">
+      <c r="F8" s="1">
         <v>21655</v>
       </c>
-      <c r="G8">
+      <c r="G8" s="1">
         <v>1271610</v>
       </c>
-      <c r="H8" s="4">
+      <c r="H8" s="1">
         <v>82.67</v>
       </c>
-      <c r="I8" s="6">
+      <c r="I8" s="3">
         <v>4.75</v>
       </c>
-      <c r="J8">
+      <c r="J8" s="1">
         <v>194.85000000000002</v>
       </c>
-      <c r="K8">
+      <c r="K8" s="1">
         <v>2.06</v>
       </c>
-    </row>
-    <row r="9" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
+      <c r="L8" s="4">
+        <v>724415.26732229581</v>
+      </c>
+      <c r="M8" s="4">
+        <v>691560.71448776871</v>
+      </c>
+      <c r="N8" s="1">
+        <v>12.52</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A9" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B9">
+      <c r="B9" s="1">
         <v>71.81</v>
       </c>
-      <c r="C9">
+      <c r="C9" s="1">
         <v>99.887090703801277</v>
       </c>
-      <c r="D9" s="3">
+      <c r="D9" s="2">
         <v>45.7</v>
       </c>
       <c r="E9" s="1">
         <v>52.17</v>
       </c>
-      <c r="F9">
+      <c r="F9" s="1">
         <v>88069</v>
       </c>
-      <c r="G9">
+      <c r="G9" s="1">
         <v>5645284</v>
       </c>
-      <c r="H9" s="4">
+      <c r="H9" s="1">
         <v>77.75</v>
       </c>
-      <c r="I9" s="6">
+      <c r="I9" s="3">
         <v>2.38</v>
       </c>
-      <c r="J9">
+      <c r="J9" s="1">
         <v>137.96</v>
       </c>
-      <c r="K9">
+      <c r="K9" s="1">
         <v>3.63</v>
       </c>
-    </row>
-    <row r="10" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
+      <c r="L9" s="4">
+        <v>656936.64990951039</v>
+      </c>
+      <c r="M9" s="4">
+        <v>544536.78550742532</v>
+      </c>
+      <c r="N9" s="1">
+        <v>10.62</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A10" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="B10">
+      <c r="B10" s="1">
         <v>73.33</v>
       </c>
-      <c r="C10">
+      <c r="C10" s="1">
         <v>100</v>
       </c>
-      <c r="D10" s="3">
+      <c r="D10" s="2">
         <v>45.59</v>
       </c>
       <c r="E10" s="1">
         <v>42.93</v>
       </c>
-      <c r="F10">
+      <c r="F10" s="1">
         <v>17721</v>
       </c>
-      <c r="G10">
+      <c r="G10" s="1">
         <v>1156989</v>
       </c>
-      <c r="H10" s="4">
+      <c r="H10" s="1">
         <v>84.83</v>
       </c>
-      <c r="I10" s="6">
+      <c r="I10" s="3">
         <v>4.18</v>
       </c>
-      <c r="J10">
+      <c r="J10" s="1">
         <v>199.78000000000003</v>
       </c>
-      <c r="K10">
+      <c r="K10" s="1">
         <v>0.79</v>
       </c>
-    </row>
-    <row r="11" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
+      <c r="L10" s="4">
+        <v>929141.91667420883</v>
+      </c>
+      <c r="M10" s="4">
+        <v>863932.17014471488</v>
+      </c>
+      <c r="N10" s="1">
+        <v>5.08</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A11" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B11">
+      <c r="B11" s="1">
         <v>77.97</v>
       </c>
-      <c r="C11">
+      <c r="C11" s="1">
         <v>100</v>
       </c>
-      <c r="D11" s="3">
+      <c r="D11" s="2">
         <v>45.43</v>
       </c>
       <c r="E11" s="1">
         <v>44.22</v>
       </c>
-      <c r="F11">
+      <c r="F11" s="1">
         <v>20444</v>
       </c>
-      <c r="G11">
+      <c r="G11" s="1">
         <v>1915667</v>
       </c>
-      <c r="H11" s="4">
+      <c r="H11" s="1">
         <v>81.09</v>
       </c>
-      <c r="I11" s="6">
+      <c r="I11" s="3">
         <v>4.3099999999999996</v>
       </c>
-      <c r="J11">
+      <c r="J11" s="1">
         <v>134.93</v>
       </c>
-      <c r="K11">
+      <c r="K11" s="1">
         <v>6.2799999999999994</v>
       </c>
-    </row>
-    <row r="12" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
+      <c r="L11" s="4">
+        <v>938634.09135863872</v>
+      </c>
+      <c r="M11" s="4">
+        <v>1170437.3698729773</v>
+      </c>
+      <c r="N11" s="1">
+        <v>4.78</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A12" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B12">
+      <c r="B12" s="1">
         <v>83.08</v>
       </c>
-      <c r="C12">
+      <c r="C12" s="1">
         <v>100</v>
       </c>
-      <c r="D12" s="3">
+      <c r="D12" s="2">
         <v>44.67</v>
       </c>
       <c r="E12" s="1">
         <v>63.54</v>
       </c>
-      <c r="F12">
+      <c r="F12" s="1">
         <v>71050</v>
       </c>
-      <c r="G12">
+      <c r="G12" s="1">
         <v>19900021</v>
       </c>
-      <c r="H12" s="4">
+      <c r="H12" s="1">
         <v>87.51</v>
       </c>
-      <c r="I12" s="6">
+      <c r="I12" s="3">
         <v>2.78</v>
       </c>
-      <c r="J12">
+      <c r="J12" s="1">
         <v>200.87</v>
       </c>
-      <c r="K12">
+      <c r="K12" s="1">
         <v>28.61</v>
       </c>
-    </row>
-    <row r="13" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
+      <c r="L12" s="4">
+        <v>1108227.6763034046</v>
+      </c>
+      <c r="M12" s="4">
+        <v>1686257.486693023</v>
+      </c>
+      <c r="N12" s="1">
+        <v>4.1399999999999997</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A13" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B13">
+      <c r="B13" s="1">
         <v>74.430000000000007</v>
       </c>
-      <c r="C13">
+      <c r="C13" s="1">
         <v>99.949639080073865</v>
       </c>
-      <c r="D13" s="3">
+      <c r="D13" s="2">
         <v>44.62</v>
       </c>
       <c r="E13" s="1">
         <v>43.38</v>
       </c>
-      <c r="F13">
+      <c r="F13" s="1">
         <v>640316</v>
       </c>
-      <c r="G13">
+      <c r="G13" s="1">
         <v>57694537</v>
       </c>
-      <c r="H13" s="4">
+      <c r="H13" s="1">
         <v>85.52</v>
       </c>
-      <c r="I13" s="6">
+      <c r="I13" s="3">
         <v>3.82</v>
       </c>
-      <c r="J13">
+      <c r="J13" s="1">
         <v>148.13</v>
       </c>
-      <c r="K13">
+      <c r="K13" s="1">
         <v>8.7899999999999991</v>
       </c>
-    </row>
-    <row r="14" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
+      <c r="L13" s="4">
+        <v>803842.31290619029</v>
+      </c>
+      <c r="M13" s="4">
+        <v>829190.14931085368</v>
+      </c>
+      <c r="N13" s="1">
+        <v>7.08</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A14" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B14">
+      <c r="B14" s="1">
         <v>73.88</v>
       </c>
-      <c r="C14">
+      <c r="C14" s="1">
         <v>99.988321849818988</v>
       </c>
-      <c r="D14" s="3">
+      <c r="D14" s="2">
         <v>44.45</v>
       </c>
       <c r="E14" s="1">
         <v>45.18</v>
       </c>
-      <c r="F14">
+      <c r="F14" s="1">
         <v>887559</v>
       </c>
-      <c r="G14">
+      <c r="G14" s="1">
         <v>46314575</v>
       </c>
-      <c r="H14" s="4">
+      <c r="H14" s="1">
         <v>81.319999999999993</v>
       </c>
-      <c r="I14" s="6">
+      <c r="I14" s="3">
         <v>2.4300000000000002</v>
       </c>
-      <c r="J14">
+      <c r="J14" s="1">
         <v>131.20999999999998</v>
       </c>
-      <c r="K14">
+      <c r="K14" s="1">
         <v>4.2</v>
       </c>
-    </row>
-    <row r="15" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
+      <c r="L14" s="4">
+        <v>647310.5091076768</v>
+      </c>
+      <c r="M14" s="4">
+        <v>624367.63041945465</v>
+      </c>
+      <c r="N14" s="1">
+        <v>9.58</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A15" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B15">
+      <c r="B15" s="1">
         <v>81.55</v>
       </c>
-      <c r="C15">
+      <c r="C15" s="1">
         <v>99.771689497716892</v>
       </c>
-      <c r="D15" s="3">
+      <c r="D15" s="2">
         <v>44.42</v>
       </c>
       <c r="E15" s="1">
         <v>56.72</v>
       </c>
-      <c r="F15">
+      <c r="F15" s="1">
         <v>125115</v>
       </c>
-      <c r="G15">
+      <c r="G15" s="1">
         <v>6032917</v>
       </c>
-      <c r="H15" s="4">
+      <c r="H15" s="1">
         <v>88.73</v>
       </c>
-      <c r="I15" s="6">
+      <c r="I15" s="3">
         <v>4.43</v>
       </c>
-      <c r="J15">
+      <c r="J15" s="1">
         <v>122.32000000000001</v>
       </c>
-      <c r="K15">
+      <c r="K15" s="1">
         <v>10.61</v>
       </c>
-    </row>
-    <row r="16" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
+      <c r="L15" s="4">
+        <v>748181.79535054578</v>
+      </c>
+      <c r="M15" s="4">
+        <v>1010682.829179725</v>
+      </c>
+      <c r="N15" s="1">
+        <v>10.4</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A16" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B16">
+      <c r="B16" s="1">
         <v>74.09</v>
       </c>
-      <c r="C16">
+      <c r="C16" s="1">
         <v>99.917588886272668</v>
       </c>
-      <c r="D16" s="3">
+      <c r="D16" s="2">
         <v>44.24</v>
       </c>
       <c r="E16" s="1">
         <v>37.54</v>
       </c>
-      <c r="F16">
+      <c r="F16" s="1">
         <v>925985</v>
       </c>
-      <c r="G16">
+      <c r="G16" s="1">
         <v>47018509</v>
       </c>
-      <c r="H16" s="4">
+      <c r="H16" s="1">
         <v>81.790000000000006</v>
       </c>
-      <c r="I16" s="6">
+      <c r="I16" s="3">
         <v>3.89</v>
       </c>
-      <c r="J16">
+      <c r="J16" s="1">
         <v>140.38</v>
       </c>
-      <c r="K16">
+      <c r="K16" s="1">
         <v>3.2300000000000004</v>
       </c>
-    </row>
-    <row r="17" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
+      <c r="L16" s="4">
+        <v>689147.65469497058</v>
+      </c>
+      <c r="M16" s="4">
+        <v>667795.59214205865</v>
+      </c>
+      <c r="N16" s="1">
+        <v>9.56</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A17" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B17">
+      <c r="B17" s="1">
         <v>74.48</v>
       </c>
-      <c r="C17">
+      <c r="C17" s="1">
         <v>99.935567010309285</v>
       </c>
-      <c r="D17" s="3">
+      <c r="D17" s="2">
         <v>44.21</v>
       </c>
       <c r="E17" s="1">
         <v>40.1</v>
       </c>
-      <c r="F17">
+      <c r="F17" s="1">
         <v>99726</v>
       </c>
-      <c r="G17">
+      <c r="G17" s="1">
         <v>8721085</v>
       </c>
-      <c r="H17" s="4">
+      <c r="H17" s="1">
         <v>84.55</v>
       </c>
-      <c r="I17" s="6">
+      <c r="I17" s="3">
         <v>3.89</v>
       </c>
-      <c r="J17">
+      <c r="J17" s="1">
         <v>141.60000000000002</v>
       </c>
-      <c r="K17">
+      <c r="K17" s="1">
         <v>15.879999999999999</v>
       </c>
-    </row>
-    <row r="18" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
+      <c r="L17" s="4">
+        <v>873268.3212992124</v>
+      </c>
+      <c r="M17" s="4">
+        <v>898893.86103886564</v>
+      </c>
+      <c r="N17" s="1">
+        <v>5.7</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A18" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B18">
+      <c r="B18" s="1">
         <v>77.760000000000005</v>
       </c>
-      <c r="C18">
+      <c r="C18" s="1">
         <v>100</v>
       </c>
-      <c r="D18" s="3">
+      <c r="D18" s="2">
         <v>44.13</v>
       </c>
       <c r="E18" s="1">
         <v>51.37</v>
       </c>
-      <c r="F18">
+      <c r="F18" s="1">
         <v>147043</v>
       </c>
-      <c r="G18">
+      <c r="G18" s="1">
         <v>6695694</v>
       </c>
-      <c r="H18" s="4">
+      <c r="H18" s="1">
         <v>85.47</v>
       </c>
-      <c r="I18" s="6">
+      <c r="I18" s="3">
         <v>3.81</v>
       </c>
-      <c r="J18">
+      <c r="J18" s="1">
         <v>168.42</v>
       </c>
-      <c r="K18">
+      <c r="K18" s="1">
         <v>4.9499999999999993</v>
       </c>
-    </row>
-    <row r="19" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
+      <c r="L18" s="4">
+        <v>804982.09674664575</v>
+      </c>
+      <c r="M18" s="4">
+        <v>1067777.5166461496</v>
+      </c>
+      <c r="N18" s="1">
+        <v>3.8</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A19" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B19">
+      <c r="B19" s="1">
         <v>70.930000000000007</v>
       </c>
-      <c r="C19">
+      <c r="C19" s="1">
         <v>99.914236706689536</v>
       </c>
-      <c r="D19" s="3">
+      <c r="D19" s="2">
         <v>43.82</v>
       </c>
       <c r="E19" s="1">
         <v>29.83</v>
       </c>
-      <c r="F19">
+      <c r="F19" s="1">
         <v>118661</v>
       </c>
-      <c r="G19">
+      <c r="G19" s="1">
         <v>5577572</v>
       </c>
-      <c r="H19" s="4">
+      <c r="H19" s="1">
         <v>66.11</v>
       </c>
-      <c r="I19" s="6">
+      <c r="I19" s="3">
         <v>2.76</v>
       </c>
-      <c r="J19">
+      <c r="J19" s="1">
         <v>219.70999999999998</v>
       </c>
-      <c r="K19">
+      <c r="K19" s="1">
         <v>1.76</v>
       </c>
-    </row>
-    <row r="20" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
+      <c r="L19" s="4">
+        <v>730070.57095624204</v>
+      </c>
+      <c r="M19" s="4">
+        <v>547068.31649781868</v>
+      </c>
+      <c r="N19" s="1">
+        <v>11.91</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A20" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B20">
+      <c r="B20" s="1">
         <v>67.39</v>
       </c>
-      <c r="C20">
+      <c r="C20" s="1">
         <v>98.784624081401915</v>
       </c>
-      <c r="D20" s="3">
+      <c r="D20" s="2">
         <v>43.59</v>
       </c>
       <c r="E20" s="1">
         <v>14.19</v>
       </c>
-      <c r="F20">
+      <c r="F20" s="1">
         <v>145293</v>
       </c>
-      <c r="G20">
+      <c r="G20" s="1">
         <v>3084108</v>
       </c>
-      <c r="H20" s="4">
+      <c r="H20" s="1">
         <v>67.75</v>
       </c>
-      <c r="I20" s="6">
+      <c r="I20" s="3">
         <v>4.0599999999999996</v>
       </c>
-      <c r="J20">
+      <c r="J20" s="1">
         <v>210.69</v>
       </c>
-      <c r="K20">
+      <c r="K20" s="1">
         <v>1.49</v>
       </c>
-    </row>
-    <row r="21" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
+      <c r="L20" s="4">
+        <v>541264.63767742424</v>
+      </c>
+      <c r="M20" s="4">
+        <v>434589.12661410269</v>
+      </c>
+      <c r="N20" s="1">
+        <v>19.02</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A21" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B21">
+      <c r="B21" s="1">
         <v>70.13</v>
       </c>
-      <c r="C21">
+      <c r="C21" s="1">
         <v>95.224849327770059</v>
       </c>
-      <c r="D21" s="3">
+      <c r="D21" s="2">
         <v>43.57</v>
       </c>
       <c r="E21" s="1">
         <v>40.020000000000003</v>
       </c>
-      <c r="F21">
+      <c r="F21" s="1">
         <v>46809</v>
       </c>
-      <c r="G21">
+      <c r="G21" s="1">
         <v>2417452</v>
       </c>
-      <c r="H21" s="4">
+      <c r="H21" s="1">
         <v>79.03</v>
       </c>
-      <c r="I21" s="6">
+      <c r="I21" s="3">
         <v>3.29</v>
       </c>
-      <c r="J21">
+      <c r="J21" s="1">
         <v>167.29000000000002</v>
       </c>
-      <c r="K21">
+      <c r="K21" s="1">
         <v>2.78</v>
       </c>
-    </row>
-    <row r="22" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
+      <c r="L21" s="4">
+        <v>735784.64013506065</v>
+      </c>
+      <c r="M21" s="4">
+        <v>652292.12554519332</v>
+      </c>
+      <c r="N21" s="1">
+        <v>6.25</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A22" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B22">
+      <c r="B22" s="1">
         <v>72.73</v>
       </c>
-      <c r="C22">
+      <c r="C22" s="1">
         <v>93.849080532656942</v>
       </c>
-      <c r="D22" s="3">
+      <c r="D22" s="2">
         <v>43.44</v>
       </c>
       <c r="E22" s="1">
         <v>35.01</v>
       </c>
-      <c r="F22">
+      <c r="F22" s="1">
         <v>29660</v>
       </c>
-      <c r="G22">
+      <c r="G22" s="1">
         <v>1218398</v>
       </c>
-      <c r="H22" s="6">
+      <c r="H22" s="3">
         <v>82.4</v>
       </c>
-      <c r="I22" s="6">
+      <c r="I22" s="3">
         <v>2.75</v>
       </c>
-      <c r="J22">
+      <c r="J22" s="1">
         <v>192.18</v>
       </c>
-      <c r="K22">
+      <c r="K22" s="1">
         <v>3.81</v>
       </c>
-    </row>
-    <row r="23" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
+      <c r="L22" s="4">
+        <v>835242.89745748928</v>
+      </c>
+      <c r="M22" s="4">
+        <v>755447.73119422246</v>
+      </c>
+      <c r="N22" s="1">
+        <v>5.26</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A23" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B23">
+      <c r="B23" s="1">
         <v>73.03</v>
       </c>
-      <c r="C23">
+      <c r="C23" s="1">
         <v>99.007444168734494</v>
       </c>
-      <c r="D23" s="3">
+      <c r="D23" s="2">
         <v>43.3</v>
       </c>
       <c r="E23" s="1">
         <v>43.43</v>
       </c>
-      <c r="F23">
+      <c r="F23" s="1">
         <v>60949</v>
       </c>
-      <c r="G23">
+      <c r="G23" s="1">
         <v>3323790</v>
       </c>
-      <c r="H23" s="4">
+      <c r="H23" s="1">
         <v>71.760000000000005</v>
       </c>
-      <c r="I23" s="6">
+      <c r="I23" s="3">
         <v>2.82</v>
       </c>
-      <c r="J23">
+      <c r="J23" s="1">
         <v>257.82</v>
       </c>
-      <c r="K23">
+      <c r="K23" s="1">
         <v>3.43</v>
       </c>
-    </row>
-    <row r="24" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A24" t="s">
+      <c r="L23" s="4">
+        <v>799947.54001444683</v>
+      </c>
+      <c r="M23" s="4">
+        <v>734091.713074642</v>
+      </c>
+      <c r="N23" s="1">
+        <v>4.0199999999999996</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A24" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B24">
+      <c r="B24" s="1">
         <v>78.83</v>
       </c>
-      <c r="C24">
+      <c r="C24" s="1">
         <v>96.292775665399247</v>
       </c>
-      <c r="D24" s="3">
+      <c r="D24" s="2">
         <v>42.86</v>
       </c>
       <c r="E24" s="1">
         <v>50.51</v>
       </c>
-      <c r="F24">
+      <c r="F24" s="1">
         <v>33551</v>
       </c>
-      <c r="G24">
+      <c r="G24" s="1">
         <v>4900061</v>
       </c>
-      <c r="H24" s="4">
+      <c r="H24" s="1">
         <v>80.63</v>
       </c>
-      <c r="I24" s="6">
+      <c r="I24" s="3">
         <v>7.46</v>
       </c>
-      <c r="J24">
+      <c r="J24" s="1">
         <v>178.63</v>
       </c>
-      <c r="K24">
+      <c r="K24" s="1">
         <v>4.1399999999999997</v>
       </c>
-    </row>
-    <row r="25" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
+      <c r="L24" s="4">
+        <v>925953.5392308631</v>
+      </c>
+      <c r="M24" s="4">
+        <v>1116837.5599591665</v>
+      </c>
+      <c r="N24" s="1">
+        <v>5.51</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A25" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B25">
+      <c r="B25" s="1">
         <v>73.02</v>
       </c>
-      <c r="C25">
+      <c r="C25" s="1">
         <v>89.049586776859499</v>
       </c>
-      <c r="D25" s="3">
+      <c r="D25" s="2">
         <v>42.32</v>
       </c>
       <c r="E25" s="1">
         <v>39.03</v>
       </c>
-      <c r="F25">
+      <c r="F25" s="1">
         <v>5953</v>
       </c>
-      <c r="G25">
+      <c r="G25" s="1">
         <v>383173</v>
       </c>
-      <c r="H25" s="4">
+      <c r="H25" s="1">
         <v>66.69</v>
       </c>
-      <c r="I25" s="6">
+      <c r="I25" s="3">
         <v>6.17</v>
       </c>
-      <c r="J25">
+      <c r="J25" s="1">
         <v>161.47999999999999</v>
       </c>
-      <c r="K25">
+      <c r="K25" s="1">
         <v>3.12</v>
       </c>
-    </row>
-    <row r="26" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A26" t="s">
+      <c r="L25" s="4">
+        <v>833208.88764531387</v>
+      </c>
+      <c r="M25" s="4">
+        <v>824833.16835916648</v>
+      </c>
+      <c r="N25" s="1">
+        <v>5.38</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A26" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B26">
+      <c r="B26" s="1">
         <v>75.03</v>
       </c>
-      <c r="C26">
+      <c r="C26" s="1">
         <v>97.878128400435259</v>
       </c>
-      <c r="D26" s="3">
+      <c r="D26" s="2">
         <v>42.26</v>
       </c>
       <c r="E26" s="1">
         <v>34.380000000000003</v>
       </c>
-      <c r="F26">
+      <c r="F26" s="1">
         <v>48901</v>
       </c>
-      <c r="G26">
+      <c r="G26" s="1">
         <v>2133442</v>
       </c>
-      <c r="H26" s="6">
+      <c r="H26" s="3">
         <v>74.2</v>
       </c>
-      <c r="I26" s="6">
+      <c r="I26" s="3">
         <v>5.35</v>
       </c>
-      <c r="J26">
+      <c r="J26" s="1">
         <v>187.05</v>
       </c>
-      <c r="K26">
+      <c r="K26" s="1">
         <v>3.33</v>
       </c>
-    </row>
-    <row r="27" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
+      <c r="L26" s="4">
+        <v>717919.36286356859</v>
+      </c>
+      <c r="M26" s="4">
+        <v>664509.7592060616</v>
+      </c>
+      <c r="N26" s="1">
+        <v>6.7</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A27" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B27">
+      <c r="B27" s="1">
         <v>71.56</v>
       </c>
-      <c r="C27">
+      <c r="C27" s="1">
         <v>98.219584569732945</v>
       </c>
-      <c r="D27" s="3">
+      <c r="D27" s="2">
         <v>42.26</v>
       </c>
       <c r="E27" s="1">
         <v>30.12</v>
       </c>
-      <c r="F27">
+      <c r="F27" s="1">
         <v>82354</v>
       </c>
-      <c r="G27">
+      <c r="G27" s="1">
         <v>4995388</v>
       </c>
-      <c r="H27" s="4">
+      <c r="H27" s="1">
         <v>60.47</v>
       </c>
-      <c r="I27" s="6">
+      <c r="I27" s="3">
         <v>2.66</v>
       </c>
-      <c r="J27">
+      <c r="J27" s="1">
         <v>179.61</v>
       </c>
-      <c r="K27">
+      <c r="K27" s="1">
         <v>1.5699999999999998</v>
       </c>
-    </row>
-    <row r="28" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A28" t="s">
+      <c r="L27" s="4">
+        <v>644418.0489760245</v>
+      </c>
+      <c r="M27" s="4">
+        <v>587035.33284214674</v>
+      </c>
+      <c r="N27" s="1">
+        <v>11.04</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A28" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B28">
+      <c r="B28" s="1">
         <v>74.05</v>
       </c>
-      <c r="C28">
+      <c r="C28" s="1">
         <v>98.921568627450981</v>
       </c>
-      <c r="D28" s="3">
+      <c r="D28" s="2">
         <v>42.07</v>
       </c>
       <c r="E28" s="1">
         <v>38.659999999999997</v>
       </c>
-      <c r="F28">
+      <c r="F28" s="1">
         <v>126803</v>
       </c>
-      <c r="G28">
+      <c r="G28" s="1">
         <v>6106779</v>
       </c>
-      <c r="H28" s="4">
+      <c r="H28" s="1">
         <v>71.81</v>
       </c>
-      <c r="I28" s="6">
+      <c r="I28" s="3">
         <v>3.02</v>
       </c>
-      <c r="J28">
+      <c r="J28" s="1">
         <v>154.51</v>
       </c>
-      <c r="K28">
+      <c r="K28" s="1">
         <v>4.3500000000000005</v>
       </c>
-    </row>
-    <row r="29" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A29" t="s">
+      <c r="L28" s="4">
+        <v>636654.75969916233</v>
+      </c>
+      <c r="M28" s="4">
+        <v>646426.25461381127</v>
+      </c>
+      <c r="N28" s="1">
+        <v>7.77</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A29" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B29">
+      <c r="B29" s="1">
         <v>73.48</v>
       </c>
-      <c r="C29">
+      <c r="C29" s="1">
         <v>97.251308900523554</v>
       </c>
-      <c r="D29" s="3">
+      <c r="D29" s="2">
         <v>41.69</v>
       </c>
       <c r="E29" s="1">
         <v>27.63</v>
       </c>
-      <c r="F29">
+      <c r="F29" s="1">
         <v>49497</v>
       </c>
-      <c r="G29">
+      <c r="G29" s="1">
         <v>6331828</v>
       </c>
-      <c r="H29" s="4">
+      <c r="H29" s="1">
         <v>64.05</v>
       </c>
-      <c r="I29" s="6">
+      <c r="I29" s="3">
         <v>5.2</v>
       </c>
-      <c r="J29">
+      <c r="J29" s="1">
         <v>168.58</v>
       </c>
-      <c r="K29">
+      <c r="K29" s="1">
         <v>2.59</v>
       </c>
-    </row>
-    <row r="30" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A30" t="s">
+      <c r="L29" s="4">
+        <v>604047.4000826244</v>
+      </c>
+      <c r="M29" s="4">
+        <v>623116.08709131391</v>
+      </c>
+      <c r="N29" s="1">
+        <v>10.63</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A30" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B30">
+      <c r="B30" s="1">
         <v>71.23</v>
       </c>
-      <c r="C30">
+      <c r="C30" s="1">
         <v>99.043715846994544</v>
       </c>
-      <c r="D30" s="3">
+      <c r="D30" s="2">
         <v>41.65</v>
       </c>
       <c r="E30" s="1">
         <v>21.37</v>
       </c>
-      <c r="F30">
+      <c r="F30" s="1">
         <v>30905</v>
       </c>
-      <c r="G30">
+      <c r="G30" s="1">
         <v>1024507</v>
       </c>
-      <c r="H30" s="4">
+      <c r="H30" s="1">
         <v>64.36</v>
       </c>
-      <c r="I30" s="6">
+      <c r="I30" s="3">
         <v>5.96</v>
       </c>
-      <c r="J30">
+      <c r="J30" s="1">
         <v>157.39000000000001</v>
       </c>
-      <c r="K30">
+      <c r="K30" s="1">
         <v>2.5300000000000002</v>
       </c>
-    </row>
-    <row r="31" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A31" t="s">
+      <c r="L30" s="4">
+        <v>620822.95769780222</v>
+      </c>
+      <c r="M30" s="4">
+        <v>641445.5230245468</v>
+      </c>
+      <c r="N30" s="1">
+        <v>13.87</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A31" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B31">
+      <c r="B31" s="1">
         <v>68.2</v>
       </c>
-      <c r="C31">
+      <c r="C31" s="1">
         <v>90.615384615384613</v>
       </c>
-      <c r="D31" s="3">
+      <c r="D31" s="2">
         <v>41.22</v>
       </c>
       <c r="E31" s="1">
         <v>28.26</v>
       </c>
-      <c r="F31">
+      <c r="F31" s="1">
         <v>24738</v>
       </c>
-      <c r="G31">
+      <c r="G31" s="1">
         <v>783884</v>
       </c>
-      <c r="H31" s="4">
+      <c r="H31" s="1">
         <v>59.11</v>
       </c>
-      <c r="I31" s="6">
+      <c r="I31" s="3">
         <v>3.55</v>
       </c>
-      <c r="J31">
+      <c r="J31" s="1">
         <v>234.03</v>
       </c>
-      <c r="K31">
+      <c r="K31" s="1">
         <v>2.54</v>
       </c>
-    </row>
-    <row r="32" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A32" t="s">
+      <c r="L31" s="4">
+        <v>579734.30313008046</v>
+      </c>
+      <c r="M31" s="4">
+        <v>529854.72641780658</v>
+      </c>
+      <c r="N31" s="1">
+        <v>10.71</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A32" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B32">
+      <c r="B32" s="1">
         <v>71.569999999999993</v>
       </c>
-      <c r="C32">
+      <c r="C32" s="1">
         <v>94.770206022187011</v>
       </c>
-      <c r="D32" s="3">
+      <c r="D32" s="2">
         <v>41.09</v>
       </c>
       <c r="E32" s="1">
         <v>31.3</v>
       </c>
-      <c r="F32">
+      <c r="F32" s="1">
         <v>43495</v>
       </c>
-      <c r="G32">
+      <c r="G32" s="1">
         <v>1025316</v>
       </c>
-      <c r="H32" s="4">
+      <c r="H32" s="1">
         <v>65.680000000000007</v>
       </c>
-      <c r="I32" s="6">
+      <c r="I32" s="3">
         <v>4.05</v>
       </c>
-      <c r="J32">
+      <c r="J32" s="1">
         <v>244.54</v>
       </c>
-      <c r="K32">
+      <c r="K32" s="1">
         <v>2.4500000000000002</v>
       </c>
-    </row>
-    <row r="33" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A33" t="s">
+      <c r="L32" s="4">
+        <v>640897.173783415</v>
+      </c>
+      <c r="M32" s="4">
+        <v>636671.86190642964</v>
+      </c>
+      <c r="N32" s="1">
+        <v>15.78</v>
+      </c>
+    </row>
+    <row r="33" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A33" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B33">
+      <c r="B33" s="1">
         <v>71.03</v>
       </c>
-      <c r="C33">
+      <c r="C33" s="1">
         <v>95.864350703060381</v>
       </c>
-      <c r="D33" s="3">
+      <c r="D33" s="2">
         <v>41.01</v>
       </c>
       <c r="E33" s="1">
         <v>21.93</v>
       </c>
-      <c r="F33">
+      <c r="F33" s="1">
         <v>15787</v>
       </c>
-      <c r="G33">
+      <c r="G33" s="1">
         <v>693628</v>
       </c>
-      <c r="H33" s="4">
+      <c r="H33" s="1">
         <v>68.45</v>
       </c>
-      <c r="I33" s="6">
+      <c r="I33" s="3">
         <v>4.0999999999999996</v>
       </c>
-      <c r="J33">
+      <c r="J33" s="1">
         <v>169.75</v>
       </c>
-      <c r="K33">
+      <c r="K33" s="1">
         <v>3.31</v>
       </c>
-    </row>
-    <row r="34" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A34" t="s">
+      <c r="L33" s="4">
+        <v>726547.04273862334</v>
+      </c>
+      <c r="M33" s="4">
+        <v>720763.29693964252</v>
+      </c>
+      <c r="N33" s="1">
+        <v>6.03</v>
+      </c>
+    </row>
+    <row r="34" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A34" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B34">
+      <c r="B34" s="1">
         <v>67.02</v>
       </c>
-      <c r="C34">
+      <c r="C34" s="1">
         <v>83.195876288659804</v>
       </c>
-      <c r="D34" s="3">
+      <c r="D34" s="2">
         <v>41</v>
       </c>
       <c r="E34" s="1">
         <v>16.09</v>
       </c>
-      <c r="F34">
+      <c r="F34" s="1">
         <v>1858</v>
       </c>
-      <c r="G34">
+      <c r="G34" s="1">
         <v>223950</v>
       </c>
-      <c r="H34" s="6">
+      <c r="H34" s="3">
         <v>75.5</v>
       </c>
-      <c r="I34" s="6">
+      <c r="I34" s="3">
         <v>6.04</v>
       </c>
-      <c r="J34">
+      <c r="J34" s="1">
         <v>230.76000000000002</v>
       </c>
-      <c r="K34">
+      <c r="K34" s="1">
         <v>5.87</v>
       </c>
-    </row>
-    <row r="35" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A35" t="s">
+      <c r="L34" s="4">
+        <v>836641.82259002433</v>
+      </c>
+      <c r="M34" s="4">
+        <v>806846.13186776266</v>
+      </c>
+      <c r="N34" s="1">
+        <v>21.09</v>
+      </c>
+    </row>
+    <row r="35" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A35" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B35">
+      <c r="B35" s="1">
         <v>68.63</v>
       </c>
-      <c r="C35">
+      <c r="C35" s="1">
         <v>92.329545454545453</v>
       </c>
-      <c r="D35" s="3">
+      <c r="D35" s="2">
         <v>40.46</v>
       </c>
       <c r="E35" s="1">
         <v>24.68</v>
       </c>
-      <c r="F35">
+      <c r="F35" s="1">
         <v>2861</v>
       </c>
-      <c r="G35">
+      <c r="G35" s="1">
         <v>272521</v>
       </c>
-      <c r="H35" s="4">
+      <c r="H35" s="1">
         <v>74.430000000000007</v>
       </c>
-      <c r="I35" s="6">
+      <c r="I35" s="3">
         <v>5.26</v>
       </c>
-      <c r="J35">
+      <c r="J35" s="1">
         <v>156.88999999999999</v>
       </c>
-      <c r="K35">
+      <c r="K35" s="1">
         <v>2.57</v>
       </c>
-    </row>
-    <row r="36" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A36" t="s">
+      <c r="L35" s="4">
+        <v>810862.59089875699</v>
+      </c>
+      <c r="M35" s="4">
+        <v>831867.44105518749</v>
+      </c>
+      <c r="N35" s="1">
+        <v>16.95</v>
+      </c>
+    </row>
+    <row r="36" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A36" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="B36">
+      <c r="B36" s="1">
         <v>73</v>
       </c>
-      <c r="C36">
+      <c r="C36" s="1">
         <v>88.046647230320701</v>
       </c>
-      <c r="D36" s="3">
+      <c r="D36" s="2">
         <v>40.11</v>
       </c>
       <c r="E36" s="1">
         <v>23.29</v>
       </c>
-      <c r="F36">
+      <c r="F36" s="1">
         <v>7499</v>
       </c>
-      <c r="G36">
+      <c r="G36" s="1">
         <v>398165</v>
       </c>
-      <c r="H36" s="4">
+      <c r="H36" s="1">
         <v>74.11</v>
       </c>
-      <c r="I36" s="6">
+      <c r="I36" s="3">
         <v>7.02</v>
       </c>
-      <c r="J36">
+      <c r="J36" s="1">
         <v>172.14</v>
       </c>
-      <c r="K36">
+      <c r="K36" s="1">
         <v>11.27</v>
       </c>
-    </row>
-    <row r="37" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A37" t="s">
+      <c r="L36" s="4">
+        <v>765392.79637549527</v>
+      </c>
+      <c r="M36" s="4">
+        <v>813501.05131505558</v>
+      </c>
+      <c r="N36" s="1">
+        <v>18.09</v>
+      </c>
+    </row>
+    <row r="37" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A37" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B37">
+      <c r="B37" s="1">
         <v>67.900000000000006</v>
       </c>
-      <c r="C37">
+      <c r="C37" s="1">
         <v>84.782608695652172</v>
       </c>
-      <c r="D37" s="3">
+      <c r="D37" s="2">
         <v>38.32</v>
       </c>
       <c r="E37" s="1">
         <v>28.98</v>
       </c>
-      <c r="F37">
+      <c r="F37" s="1">
         <v>4931</v>
       </c>
-      <c r="G37">
+      <c r="G37" s="1">
         <v>363652</v>
       </c>
-      <c r="H37" s="4">
+      <c r="H37" s="1">
         <v>73.209999999999994</v>
       </c>
-      <c r="I37" s="6">
+      <c r="I37" s="3">
         <v>2.91</v>
       </c>
-      <c r="J37">
+      <c r="J37" s="1">
         <v>236.01</v>
       </c>
-      <c r="K37">
+      <c r="K37" s="1">
         <v>1.29</v>
       </c>
-    </row>
-    <row r="38" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A38" t="s">
+      <c r="L37" s="4">
+        <v>749474.4527901751</v>
+      </c>
+      <c r="M37" s="4">
+        <v>677615.67825113039</v>
+      </c>
+      <c r="N37" s="1">
+        <v>19.350000000000001</v>
+      </c>
+    </row>
+    <row r="38" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A38" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="B38">
+      <c r="B38" s="1">
         <v>59.75</v>
       </c>
-      <c r="C38">
+      <c r="C38" s="1">
         <v>27.897350993377483</v>
       </c>
-      <c r="D38" s="3">
+      <c r="D38" s="2">
         <v>36.659999999999997</v>
       </c>
       <c r="E38" s="1">
         <v>28.78</v>
       </c>
-      <c r="F38">
+      <c r="F38" s="1">
         <v>3828</v>
       </c>
-      <c r="G38">
+      <c r="G38" s="1">
         <v>290986</v>
       </c>
-      <c r="H38" s="4">
+      <c r="H38" s="1">
         <v>73.28</v>
       </c>
-      <c r="I38" s="6">
+      <c r="I38" s="3">
         <v>0.56000000000000005</v>
       </c>
-      <c r="J38">
+      <c r="J38" s="1">
         <v>156.26</v>
       </c>
-      <c r="K38">
+      <c r="K38" s="1">
         <v>1.75</v>
       </c>
-    </row>
-    <row r="39" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A39" t="s">
+      <c r="L38" s="4">
+        <v>887039.15923625638</v>
+      </c>
+      <c r="M38" s="4">
+        <v>600648.7380136404</v>
+      </c>
+      <c r="N38" s="1">
+        <v>27.6</v>
+      </c>
+    </row>
+    <row r="39" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A39" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B39">
+      <c r="B39" s="1">
         <v>53.42</v>
       </c>
-      <c r="C39">
+      <c r="C39" s="1">
         <v>36.712224753227026</v>
       </c>
-      <c r="D39" s="3">
+      <c r="D39" s="2">
         <v>32.479999999999997</v>
       </c>
       <c r="E39" s="1">
         <v>2.7</v>
       </c>
-      <c r="F39">
+      <c r="F39" s="1">
         <v>587</v>
       </c>
-      <c r="G39">
+      <c r="G39" s="1">
         <v>51030</v>
       </c>
-      <c r="H39" s="5">
+      <c r="H39" s="1">
         <v>57.3</v>
       </c>
-      <c r="I39" s="6">
+      <c r="I39" s="3">
         <v>2.89</v>
       </c>
-      <c r="J39">
+      <c r="J39" s="1">
         <v>151.42000000000002</v>
       </c>
-      <c r="K39">
+      <c r="K39" s="1">
         <v>0</v>
+      </c>
+      <c r="L39" s="4">
+        <v>1157570.7556626785</v>
+      </c>
+      <c r="M39" s="4">
+        <v>570904.33318308706</v>
+      </c>
+      <c r="N39" s="1">
+        <v>29.66</v>
       </c>
     </row>
   </sheetData>

</xml_diff>